<commit_message>
Milestone 2: student portfolio with goals, targets, check-ins, results and photos
- Child-friendly home page with six section tiles and progress
- Answers saved one row per response; check-ins cannot be changed once sent
- Score targets for WA2, each refused by the server without a process goal
- Gap reflections on WA1 results; photo upload to a private Drive folder
- Placeholder keyword safety scan on sensitive prompts
- Students see Released feedback only
- 12 new automated tests

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017kPEbgFP64HoGA6bDARMMo
</commit_message>
<xml_diff>
--- a/seed/PHPPS_Portfolio_Data.xlsx
+++ b/seed/PHPPS_Portfolio_Data.xlsx
@@ -3473,7 +3473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I313"/>
+  <dimension ref="A1:I319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16262,6 +16262,252 @@
         </is>
       </c>
       <c r="I313" t="inlineStr">
+        <is>
+          <t>Not needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>R00313</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>S2027-0001</t>
+        </is>
+      </c>
+      <c r="C314" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Term 1 end</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>GR01</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>EV001</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr"/>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>2027-03-08 11:20</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>Not needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>R00314</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>S2027-0003</t>
+        </is>
+      </c>
+      <c r="C315" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Term 1 end</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>GR01</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>EV002</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr"/>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>2027-03-17 15:41</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>Not needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>R00315</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>S2027-0005</t>
+        </is>
+      </c>
+      <c r="C316" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Term 1 end</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>GR01</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>EV003</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr"/>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>2027-03-06 13:12</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>Not needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>R00316</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>S2027-0010</t>
+        </is>
+      </c>
+      <c r="C317" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Term 1 end</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>GR01</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>EV004</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr"/>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>2027-03-15 11:58</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>Not needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>R00317</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>S2027-0014</t>
+        </is>
+      </c>
+      <c r="C318" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Term 1 end</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>GR01</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>EV005</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr"/>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>2027-03-09 15:05</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>Not needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>R00318</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>S2027-0020</t>
+        </is>
+      </c>
+      <c r="C319" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Term 1 end</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>GR01</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>EV006</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr"/>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>2027-03-04 10:12</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr">
         <is>
           <t>Not needed</t>
         </is>

</xml_diff>